<commit_message>
Substitui dados de testes por exemplos totalmente fictícios no RPA SISREG v0.2
</commit_message>
<xml_diff>
--- a/tests/fixtures/hospital_sintetico.xlsx
+++ b/tests/fixtures/hospital_sintetico.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="POA CIRURGICO" sheetId="1" r:id="R76733ed61e314fdf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PT6" sheetId="2" r:id="R14bd2cb9f543407d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ALTA COMPLEXIDADE" sheetId="3" r:id="Re37f86c649a94428"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="POA CIRURGICO" sheetId="1" r:id="R6a35b41007144454"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PT6" sheetId="2" r:id="Rd589079cb9e74bdd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ALTA COMPLEXIDADE" sheetId="3" r:id="R6125b3cc59314c21"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -299,7 +299,7 @@
         <x:v>ANA MARIA</x:v>
       </x:c>
       <x:c r="B2" t="str">
-        <x:v>4226500330294</x:v>
+        <x:v>9000000000123</x:v>
       </x:c>
       <x:c r="C2" t="str">
         <x:v>0408050063</x:v>

</xml_diff>